<commit_message>
Change booking window rule to +7 months → first Sunday of next month
Old rule: Gate Day → Sunday of the week containing (Gate+6mo).
New rule: Gate Day → first Sunday of the month after (Gate+7mo).

Examples (verified):
  Gate 2026-05-02 → 2027-01-03  (was 2026-11-08)
  Gate 2026-12-05 → 2027-08-01  (was 2027-06-06)

Also fixes a latent timezone off-by-one in the iso() helper of
roundWindow: toISOString().slice(0,10) returns the UTC date, which in
UTC+ timezones (e.g. Asia/Taipei) rolled the displayed end date back by
one day. Switched to a local-date formatter consistent with the rest of
the file.

Updated booking_rules.md, the help text in the manager block, and the
make_tests.py F6 boundary case (2027-06-04 → 2027-08-02) so the test
batches still exercise the "迄日晚於本輪結束" reject path under the new
window. Regenerated batch-*.xlsx accordingly.

https://claude.ai/code/session_01Xvv7B8A2RUtAptByZEv9ao
</commit_message>
<xml_diff>
--- a/batch-2027-04.xlsx
+++ b/batch-2027-04.xlsx
@@ -587,12 +587,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2027-06-04</t>
+          <t>2027-08-02</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2027-06-10</t>
+          <t>2027-08-06</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -868,16 +868,16 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2027-06-04</t>
+          <t>2027-08-02</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2027-06-10</t>
+          <t>2027-08-06</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Revert "Merge pull request #2 from Evelyn68961/claude/fix-booking-date-range-a33Eq"
This reverts commit fa50258700b5c42e2c8f1f47d647ee4cbd0160cf, reversing
changes made to 97661ed10258acdfcf34e8a4d07bd98e391eaf84.
</commit_message>
<xml_diff>
--- a/batch-2027-04.xlsx
+++ b/batch-2027-04.xlsx
@@ -587,12 +587,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2027-08-02</t>
+          <t>2027-06-04</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2027-08-06</t>
+          <t>2027-06-10</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -868,16 +868,16 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2027-08-02</t>
+          <t>2027-06-04</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2027-08-06</t>
+          <t>2027-06-10</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>

</xml_diff>